<commit_message>
Fix Croquis Err510 and add fixed GPM design-flow override
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/sanitary-pumping/sanitary_pump_preliminary_design.xlsx
+++ b/engineering/sanitary-pumping/sanitary_pump_preliminary_design.xlsx
@@ -692,7 +692,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -895,7 +895,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1134,7 +1134,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1221,7 +1221,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1254,7 +1254,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -1996,9 +1996,68 @@
       </c>
     </row>
     <row r="13" ht="21" customHeight="1" s="32"/>
-    <row r="14" ht="21" customHeight="1" s="32"/>
-    <row r="15" ht="21" customHeight="1" s="32"/>
-    <row r="16" ht="21" customHeight="1" s="32"/>
+    <row r="14" ht="21" customHeight="1" s="32">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Fixed total design inflow override</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>US gpm</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="inlineStr">
+        <is>
+          <t>If &gt;0, this value overrides computed average and peak inflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1" s="32">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>Equivalent fixed inflow</t>
+        </is>
+      </c>
+      <c r="B15" s="43">
+        <f>IF(B14&gt;0,B14*0.0630902,"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>L/s</t>
+        </is>
+      </c>
+      <c r="D15" s="39" t="inlineStr">
+        <is>
+          <t>Reference conversion (1 US gpm = 0.0630902 L/s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="21" customHeight="1" s="32">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>Equivalent daily volume</t>
+        </is>
+      </c>
+      <c r="B16" s="43">
+        <f>IF(B14&gt;0,B14*5.45099,"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>m3/d</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="inlineStr">
+        <is>
+          <t>Reference conversion (1 US gpm = 5.45099 m3/d).</t>
+        </is>
+      </c>
+    </row>
     <row r="17" ht="21" customHeight="1" s="32"/>
     <row r="18" ht="21" customHeight="1" s="32">
       <c r="A18" s="41" t="inlineStr">
@@ -2632,7 +2691,7 @@
         </is>
       </c>
       <c r="B6" s="45">
-        <f>(B4+B5+Inputs!B9)*Inputs!F35</f>
+        <f>IF(Inputs!B14&gt;0,Inputs!B14*5.45099,(B4+B5+Inputs!B9)*Inputs!F35)</f>
         <v/>
       </c>
       <c r="C6" s="37" t="inlineStr">
@@ -2640,9 +2699,9 @@
           <t>m3/d</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Includes future-flow factor.</t>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>If fixed GPM override is entered, average flow follows override conversion.</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -2672,12 +2731,17 @@
         </is>
       </c>
       <c r="B7" s="45">
-        <f>B6*Inputs!B10*1000/86400*Inputs!B12</f>
+        <f>IF(Inputs!B14&gt;0,Inputs!B14*0.0630902,B6*Inputs!B10*1000/86400*Inputs!B12)</f>
         <v/>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
           <t>L/s</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>If fixed GPM override is entered, peak flow uses override directly.</t>
         </is>
       </c>
       <c r="E7" s="37" t="inlineStr">
@@ -3127,7 +3191,7 @@
           <t>L/s</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="31" t="inlineStr">
         <is>
           <t>Closest intersection between trial pump and system curves.</t>
         </is>
@@ -3202,7 +3266,7 @@
           <t>kW</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="31" t="inlineStr">
         <is>
           <t>Preliminary motor sizing check.</t>
         </is>
@@ -3242,7 +3306,7 @@
           <t>m</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="31" t="inlineStr">
         <is>
           <t>Absolute value near zero indicates good match.</t>
         </is>
@@ -4657,27 +4721,31 @@
     <row r="10" ht="21" customHeight="1" s="32">
       <c r="B10" s="61" t="n"/>
       <c r="F10" s="62" t="n"/>
-      <c r="G10" s="66">
-        <f>&gt;</f>
-        <v/>
+      <c r="G10" s="66" t="inlineStr">
+        <is>
+          <t>-&gt;</t>
+        </is>
       </c>
       <c r="H10" s="61" t="n"/>
       <c r="L10" s="62" t="n"/>
-      <c r="M10" s="66">
-        <f>&gt;</f>
-        <v/>
+      <c r="M10" s="66" t="inlineStr">
+        <is>
+          <t>-&gt;</t>
+        </is>
       </c>
       <c r="N10" s="61" t="n"/>
       <c r="R10" s="62" t="n"/>
-      <c r="S10" s="66">
-        <f>&gt;</f>
-        <v/>
+      <c r="S10" s="66" t="inlineStr">
+        <is>
+          <t>-&gt;</t>
+        </is>
       </c>
       <c r="T10" s="61" t="n"/>
       <c r="X10" s="62" t="n"/>
-      <c r="Y10" s="66">
-        <f>&gt;</f>
-        <v/>
+      <c r="Y10" s="66" t="inlineStr">
+        <is>
+          <t>-&gt;</t>
+        </is>
       </c>
       <c r="Z10" s="61" t="n"/>
       <c r="AD10" s="62" t="n"/>
@@ -4821,16 +4889,16 @@
       </c>
     </row>
     <row r="20" ht="21" customHeight="1" s="32">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Industrial area used in sizing is fixed external assumption.</t>
         </is>
       </c>
-      <c r="B20">
+      <c r="B20" s="31">
         <f>Inputs!B29</f>
         <v/>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
@@ -4951,7 +5019,6 @@
     <row r="79" ht="21" customHeight="1" s="32"/>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="N20:P20"/>
     <mergeCell ref="H7:L14"/>
     <mergeCell ref="T19:V19"/>
     <mergeCell ref="B7:F14"/>
@@ -4961,9 +5028,10 @@
     <mergeCell ref="N18:P18"/>
     <mergeCell ref="N22:P22"/>
     <mergeCell ref="B17:D17"/>
+    <mergeCell ref="T21:V21"/>
     <mergeCell ref="T17:V17"/>
-    <mergeCell ref="T21:V21"/>
     <mergeCell ref="H17:J17"/>
+    <mergeCell ref="N20:P20"/>
     <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Add office land-use inputs and link office flow to design total
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/sanitary-pumping/sanitary_pump_preliminary_design.xlsx
+++ b/engineering/sanitary-pumping/sanitary_pump_preliminary_design.xlsx
@@ -1995,7 +1995,26 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="21" customHeight="1" s="32"/>
+    <row r="13" ht="21" customHeight="1" s="32">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>Office contributing area</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="inlineStr">
+        <is>
+          <t>Office floor area connected to sanitary system.</t>
+        </is>
+      </c>
+    </row>
     <row r="14" ht="21" customHeight="1" s="32">
       <c r="A14" s="37" t="inlineStr">
         <is>
@@ -2012,7 +2031,7 @@
       </c>
       <c r="D14" s="39" t="inlineStr">
         <is>
-          <t>If &gt;0, this value overrides computed average and peak inflow.</t>
+          <t>If &gt;0, this value overrides computed average and peak inflow (including office/employee/process inputs).</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2077,26 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="21" customHeight="1" s="32"/>
+    <row r="17" ht="21" customHeight="1" s="32">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>Office wastewater allowance by area</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>L/m2/d</t>
+        </is>
+      </c>
+      <c r="D17" s="39" t="inlineStr">
+        <is>
+          <t>Preliminary office land-use unit flow; replace with local criterion if available.</t>
+        </is>
+      </c>
+    </row>
     <row r="18" ht="21" customHeight="1" s="32">
       <c r="A18" s="41" t="inlineStr">
         <is>
@@ -2581,7 +2619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="31" min="1" max="1"/>
@@ -2617,7 +2655,7 @@
     <row r="4" ht="21" customHeight="1" s="32">
       <c r="A4" s="37" t="inlineStr">
         <is>
-          <t>Area-based flow</t>
+          <t>Industrial area-based flow</t>
         </is>
       </c>
       <c r="B4" s="44">
@@ -2669,6 +2707,11 @@
           <t>m3/d</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fixtures/staff domestic component.</t>
+        </is>
+      </c>
       <c r="E5" s="37" t="inlineStr">
         <is>
           <t>Active wet-well volume</t>
@@ -2691,7 +2734,7 @@
         </is>
       </c>
       <c r="B6" s="45">
-        <f>IF(Inputs!B14&gt;0,Inputs!B14*5.45099,(B4+B5+Inputs!B9)*Inputs!F35)</f>
+        <f>IF(Inputs!B14&gt;0,Inputs!B14*5.45099,(B4+B5+B39+Inputs!B9)*Inputs!F35)</f>
         <v/>
       </c>
       <c r="C6" s="37" t="inlineStr">
@@ -2701,7 +2744,7 @@
       </c>
       <c r="D6" s="31" t="inlineStr">
         <is>
-          <t>If fixed GPM override is entered, average flow follows override conversion.</t>
+          <t>Includes industrial + office area flow + employee + process, with future-flow factor.</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -2739,7 +2782,7 @@
           <t>L/s</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>If fixed GPM override is entered, peak flow uses override directly.</t>
         </is>
@@ -3479,7 +3522,27 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="21" customHeight="1" s="32"/>
+    <row r="39" ht="21" customHeight="1" s="32">
+      <c r="A39" s="37" t="inlineStr">
+        <is>
+          <t>Office area-based flow</t>
+        </is>
+      </c>
+      <c r="B39" s="45">
+        <f>Inputs!B13*Inputs!B17/1000</f>
+        <v/>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>m3/d</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>Added to total average flow when override is off.</t>
+        </is>
+      </c>
+    </row>
     <row r="40" ht="21" customHeight="1" s="32"/>
     <row r="41" ht="21" customHeight="1" s="32"/>
     <row r="42" ht="21" customHeight="1" s="32"/>
@@ -5028,9 +5091,9 @@
     <mergeCell ref="N18:P18"/>
     <mergeCell ref="N22:P22"/>
     <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="T17:V17"/>
     <mergeCell ref="T21:V21"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="H17:J17"/>
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="A1:AD1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add cafeteria occupancy-to-DFU design module and flow integration
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/sanitary-pumping/sanitary_pump_preliminary_design.xlsx
+++ b/engineering/sanitary-pumping/sanitary_pump_preliminary_design.xlsx
@@ -1650,13 +1650,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="48" customWidth="1" style="31" min="1" max="1"/>
+    <col width="58" customWidth="1" style="31" min="1" max="1"/>
     <col width="15" customWidth="1" style="31" min="2" max="2"/>
     <col width="10" customWidth="1" style="31" min="3" max="3"/>
-    <col width="60" customWidth="1" style="31" min="4" max="4"/>
+    <col width="68" customWidth="1" style="31" min="4" max="4"/>
     <col width="40" customWidth="1" style="31" min="5" max="5"/>
     <col width="16" customWidth="1" style="31" min="6" max="6"/>
     <col width="12" customWidth="1" style="31" min="7" max="7"/>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D14" s="39" t="inlineStr">
         <is>
-          <t>If &gt;0, this value overrides computed average and peak inflow (including office/employee/process inputs).</t>
+          <t>If &gt;0, this value overrides computed average and peak inflow (industrial/office/cafeteria/employee/process).</t>
         </is>
       </c>
     </row>
@@ -2554,33 +2554,539 @@
       </c>
     </row>
     <row r="36" ht="21" customHeight="1" s="32"/>
-    <row r="37" ht="21" customHeight="1" s="32"/>
-    <row r="38" ht="21" customHeight="1" s="32"/>
-    <row r="39" ht="21" customHeight="1" s="32"/>
-    <row r="40" ht="21" customHeight="1" s="32"/>
-    <row r="41" ht="21" customHeight="1" s="32"/>
-    <row r="42" ht="21" customHeight="1" s="32"/>
-    <row r="43" ht="21" customHeight="1" s="32"/>
-    <row r="44" ht="21" customHeight="1" s="32"/>
-    <row r="45" ht="21" customHeight="1" s="32"/>
-    <row r="46" ht="21" customHeight="1" s="32"/>
-    <row r="47" ht="21" customHeight="1" s="32"/>
-    <row r="48" ht="21" customHeight="1" s="32"/>
-    <row r="49" ht="21" customHeight="1" s="32"/>
-    <row r="50" ht="21" customHeight="1" s="32"/>
-    <row r="51" ht="21" customHeight="1" s="32"/>
-    <row r="52" ht="21" customHeight="1" s="32"/>
-    <row r="53" ht="21" customHeight="1" s="32"/>
-    <row r="54" ht="21" customHeight="1" s="32"/>
-    <row r="55" ht="21" customHeight="1" s="32"/>
-    <row r="56" ht="21" customHeight="1" s="32"/>
-    <row r="57" ht="21" customHeight="1" s="32"/>
-    <row r="58" ht="21" customHeight="1" s="32"/>
-    <row r="59" ht="21" customHeight="1" s="32"/>
-    <row r="60" ht="21" customHeight="1" s="32"/>
-    <row r="61" ht="21" customHeight="1" s="32"/>
-    <row r="62" ht="21" customHeight="1" s="32"/>
-    <row r="63" ht="21" customHeight="1" s="32"/>
+    <row r="37" ht="21" customHeight="1" s="32">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>Cafeteria / Food-Service Code Module (Area -&gt; Occupants -&gt; Fixtures -&gt; DFU)</t>
+        </is>
+      </c>
+      <c r="B37" s="40" t="n"/>
+      <c r="C37" s="37" t="n"/>
+      <c r="D37" s="39" t="n"/>
+    </row>
+    <row r="38" ht="21" customHeight="1" s="32">
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>Cafeteria floor area</t>
+        </is>
+      </c>
+      <c r="B38" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="37" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D38" s="39" t="inlineStr">
+        <is>
+          <t>Dining/serving area connected to sanitary system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="21" customHeight="1" s="32">
+      <c r="A39" s="37" t="inlineStr">
+        <is>
+          <t>Occupant load factor</t>
+        </is>
+      </c>
+      <c r="B39" s="43" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>m2/person</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>Set per applicable building-code occupancy table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="21" customHeight="1" s="32">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>Calculated cafeteria occupants</t>
+        </is>
+      </c>
+      <c r="B40" s="43">
+        <f>IF(OR(B38&lt;=0,B39&lt;=0),"",ROUNDUP(B38/B39,0))</f>
+        <v/>
+      </c>
+      <c r="C40" s="37" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="D40" s="39" t="inlineStr">
+        <is>
+          <t>Based on area and occupant-load factor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="21" customHeight="1" s="32">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>Male fraction of occupants</t>
+        </is>
+      </c>
+      <c r="B41" s="43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Adjust if known; otherwise 50/50 preliminary split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="21" customHeight="1" s="32">
+      <c r="A42" s="37" t="inlineStr">
+        <is>
+          <t>Female fraction of occupants</t>
+        </is>
+      </c>
+      <c r="B42" s="43">
+        <f>IF(B41="","",1-B41)</f>
+        <v/>
+      </c>
+      <c r="C42" s="37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="39" t="inlineStr">
+        <is>
+          <t>Auto from male fraction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="21" customHeight="1" s="32">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>Male occupants (cafeteria)</t>
+        </is>
+      </c>
+      <c r="B43" s="43">
+        <f>IF(B40="","",ROUNDUP(B40*B41,0))</f>
+        <v/>
+      </c>
+      <c r="C43" s="37" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="D43" s="39" t="inlineStr">
+        <is>
+          <t>Rounded up for conservative fixture checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="21" customHeight="1" s="32">
+      <c r="A44" s="37" t="inlineStr">
+        <is>
+          <t>Female occupants (cafeteria)</t>
+        </is>
+      </c>
+      <c r="B44" s="43">
+        <f>IF(B40="","",B40-B43)</f>
+        <v/>
+      </c>
+      <c r="C44" s="37" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="D44" s="39" t="inlineStr">
+        <is>
+          <t>Balance of total occupants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="21" customHeight="1" s="32">
+      <c r="A45" s="37" t="inlineStr">
+        <is>
+          <t>Design criterion: persons per WC (men)</t>
+        </is>
+      </c>
+      <c r="B45" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="C45" s="37" t="inlineStr">
+        <is>
+          <t>pers/WC</t>
+        </is>
+      </c>
+      <c r="D45" s="39" t="inlineStr">
+        <is>
+          <t>Set from Chapter I sanitary-facility table or AHJ requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="21" customHeight="1" s="32">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>Design criterion: persons per WC (women)</t>
+        </is>
+      </c>
+      <c r="B46" s="43" t="n">
+        <v>25</v>
+      </c>
+      <c r="C46" s="37" t="inlineStr">
+        <is>
+          <t>pers/WC</t>
+        </is>
+      </c>
+      <c r="D46" s="39" t="inlineStr">
+        <is>
+          <t>Set from Chapter I sanitary-facility table or AHJ requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="21" customHeight="1" s="32">
+      <c r="A47" s="37" t="inlineStr">
+        <is>
+          <t>Design criterion: persons per urinal (men)</t>
+        </is>
+      </c>
+      <c r="B47" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="C47" s="37" t="inlineStr">
+        <is>
+          <t>pers/urinal</t>
+        </is>
+      </c>
+      <c r="D47" s="39" t="inlineStr">
+        <is>
+          <t>Set to 0 if urinals not permitted/used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="21" customHeight="1" s="32">
+      <c r="A48" s="37" t="inlineStr">
+        <is>
+          <t>Design criterion: persons per lavatory (each sex)</t>
+        </is>
+      </c>
+      <c r="B48" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="C48" s="37" t="inlineStr">
+        <is>
+          <t>pers/lav</t>
+        </is>
+      </c>
+      <c r="D48" s="39" t="inlineStr">
+        <is>
+          <t>Project/AHJ criterion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="21" customHeight="1" s="32">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>Required WCs (men)</t>
+        </is>
+      </c>
+      <c r="B49" s="43">
+        <f>IF(OR(B43="",B45&lt;=0),"",MAX(1,ROUNDUP(B43/B45,0)))</f>
+        <v/>
+      </c>
+      <c r="C49" s="37" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D49" s="39" t="inlineStr">
+        <is>
+          <t>Minimum fixture count estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="21" customHeight="1" s="32">
+      <c r="A50" s="37" t="inlineStr">
+        <is>
+          <t>Required WCs (women)</t>
+        </is>
+      </c>
+      <c r="B50" s="43">
+        <f>IF(OR(B44="",B46&lt;=0),"",MAX(1,ROUNDUP(B44/B46,0)))</f>
+        <v/>
+      </c>
+      <c r="C50" s="37" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D50" s="39" t="inlineStr">
+        <is>
+          <t>Minimum fixture count estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="21" customHeight="1" s="32">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>Required urinals (men)</t>
+        </is>
+      </c>
+      <c r="B51" s="43">
+        <f>IF(OR(B43="",B47&lt;=0),0,ROUNDUP(B43/B47,0))</f>
+        <v/>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>Set criterion per authority; can be zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="21" customHeight="1" s="32">
+      <c r="A52" s="37" t="inlineStr">
+        <is>
+          <t>Required lavatories (men)</t>
+        </is>
+      </c>
+      <c r="B52" s="43">
+        <f>IF(OR(B43="",B48&lt;=0),"",MAX(1,ROUNDUP(B43/B48,0)))</f>
+        <v/>
+      </c>
+      <c r="C52" s="37" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D52" s="39" t="inlineStr">
+        <is>
+          <t>Minimum fixture count estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="21" customHeight="1" s="32">
+      <c r="A53" s="37" t="inlineStr">
+        <is>
+          <t>Required lavatories (women)</t>
+        </is>
+      </c>
+      <c r="B53" s="43">
+        <f>IF(OR(B44="",B48&lt;=0),"",MAX(1,ROUNDUP(B44/B48,0)))</f>
+        <v/>
+      </c>
+      <c r="C53" s="37" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D53" s="39" t="inlineStr">
+        <is>
+          <t>Minimum fixture count estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="21" customHeight="1" s="32">
+      <c r="A54" s="41" t="inlineStr">
+        <is>
+          <t>DFU factors per fixture (Chapter III / NPC tables)</t>
+        </is>
+      </c>
+      <c r="B54" s="40" t="n"/>
+      <c r="C54" s="37" t="n"/>
+      <c r="D54" s="39" t="n"/>
+    </row>
+    <row r="55" ht="21" customHeight="1" s="32">
+      <c r="A55" s="37" t="inlineStr">
+        <is>
+          <t>DFU per WC</t>
+        </is>
+      </c>
+      <c r="B55" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" s="37" t="inlineStr">
+        <is>
+          <t>FU/u</t>
+        </is>
+      </c>
+      <c r="D55" s="39" t="inlineStr">
+        <is>
+          <t>Typical WC with flush tank; confirm fixture type and table value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="21" customHeight="1" s="32">
+      <c r="A56" s="37" t="inlineStr">
+        <is>
+          <t>DFU per urinal</t>
+        </is>
+      </c>
+      <c r="B56" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="37" t="inlineStr">
+        <is>
+          <t>FU/u</t>
+        </is>
+      </c>
+      <c r="D56" s="39" t="inlineStr">
+        <is>
+          <t>Depends on urinal type per Table 2.4.9.3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="21" customHeight="1" s="32">
+      <c r="A57" s="37" t="inlineStr">
+        <is>
+          <t>DFU per lavatory</t>
+        </is>
+      </c>
+      <c r="B57" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>FU/u</t>
+        </is>
+      </c>
+      <c r="D57" s="39" t="inlineStr">
+        <is>
+          <t>Lavatory DFU per applicable table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="21" customHeight="1" s="32">
+      <c r="A58" s="37" t="inlineStr">
+        <is>
+          <t>Cafeteria total DFU</t>
+        </is>
+      </c>
+      <c r="B58" s="43">
+        <f>B49*B55+B50*B55+B51*B56+B52*B57+B53*B57</f>
+        <v/>
+      </c>
+      <c r="C58" s="37" t="inlineStr">
+        <is>
+          <t>FU</t>
+        </is>
+      </c>
+      <c r="D58" s="39" t="inlineStr">
+        <is>
+          <t>Total sanitary hydraulic load from estimated fixture counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="21" customHeight="1" s="32">
+      <c r="A59" s="37" t="inlineStr">
+        <is>
+          <t>Hydraulic load equivalent (NPC 2.4.10.5)</t>
+        </is>
+      </c>
+      <c r="B59" s="43">
+        <f>IF(B58="","",IF(B58&lt;=260,2360,9.1*B58))</f>
+        <v/>
+      </c>
+      <c r="C59" s="37" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D59" s="39" t="inlineStr">
+        <is>
+          <t>Equivalent load in litres from fixture units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="21" customHeight="1" s="32">
+      <c r="A60" s="37" t="inlineStr">
+        <is>
+          <t>Assumed discharge duration for equivalent peak</t>
+        </is>
+      </c>
+      <c r="B60" s="43" t="n">
+        <v>900</v>
+      </c>
+      <c r="C60" s="37" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="D60" s="39" t="inlineStr">
+        <is>
+          <t>Use engineering judgment; 900 s = 15 minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="21" customHeight="1" s="32">
+      <c r="A61" s="37" t="inlineStr">
+        <is>
+          <t>Equivalent cafeteria peak flow from DFU</t>
+        </is>
+      </c>
+      <c r="B61" s="43">
+        <f>IF(OR(B59="",B60&lt;=0),"",B59/B60)</f>
+        <v/>
+      </c>
+      <c r="C61" s="37" t="inlineStr">
+        <is>
+          <t>L/s</t>
+        </is>
+      </c>
+      <c r="D61" s="39" t="inlineStr">
+        <is>
+          <t>Used as a code-based peak check in Design Summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="21" customHeight="1" s="32">
+      <c r="A62" s="37" t="inlineStr">
+        <is>
+          <t>Unit wastewater flow per cafeteria occupant</t>
+        </is>
+      </c>
+      <c r="B62" s="43" t="n">
+        <v>35</v>
+      </c>
+      <c r="C62" s="37" t="inlineStr">
+        <is>
+          <t>L/p/d</t>
+        </is>
+      </c>
+      <c r="D62" s="39" t="inlineStr">
+        <is>
+          <t>Set from local wastewater guidance or measured data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="21" customHeight="1" s="32">
+      <c r="A63" s="37" t="inlineStr">
+        <is>
+          <t>Cafeteria average daily flow</t>
+        </is>
+      </c>
+      <c r="B63" s="43">
+        <f>IF(B40="","",B40*B62/1000)</f>
+        <v/>
+      </c>
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>m3/d</t>
+        </is>
+      </c>
+      <c r="D63" s="39" t="inlineStr">
+        <is>
+          <t>Added to total average flow when fixed GPM override is off.</t>
+        </is>
+      </c>
+    </row>
     <row r="64" ht="21" customHeight="1" s="32"/>
     <row r="65" ht="21" customHeight="1" s="32"/>
     <row r="66" ht="21" customHeight="1" s="32"/>
@@ -2619,7 +3125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="31" min="1" max="1"/>
@@ -2707,7 +3213,7 @@
           <t>m3/d</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="31" t="inlineStr">
         <is>
           <t>Fixtures/staff domestic component.</t>
         </is>
@@ -2734,7 +3240,7 @@
         </is>
       </c>
       <c r="B6" s="45">
-        <f>IF(Inputs!B14&gt;0,Inputs!B14*5.45099,(B4+B5+B39+Inputs!B9)*Inputs!F35)</f>
+        <f>IF(Inputs!B14&gt;0,Inputs!B14*5.45099,(B4+B5+B39+B40+Inputs!B9)*Inputs!F35)</f>
         <v/>
       </c>
       <c r="C6" s="37" t="inlineStr">
@@ -2744,7 +3250,7 @@
       </c>
       <c r="D6" s="31" t="inlineStr">
         <is>
-          <t>Includes industrial + office area flow + employee + process, with future-flow factor.</t>
+          <t>Includes industrial + office + cafeteria + employee + process, with future-flow factor.</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -2774,7 +3280,7 @@
         </is>
       </c>
       <c r="B7" s="45">
-        <f>IF(Inputs!B14&gt;0,Inputs!B14*0.0630902,B6*Inputs!B10*1000/86400*Inputs!B12)</f>
+        <f>IF(Inputs!B14&gt;0,Inputs!B14*0.0630902,MAX(B6*Inputs!B10*1000/86400*Inputs!B12,IF(B41="",0,B41)))</f>
         <v/>
       </c>
       <c r="C7" s="37" t="inlineStr">
@@ -2784,7 +3290,7 @@
       </c>
       <c r="D7" s="31" t="inlineStr">
         <is>
-          <t>If fixed GPM override is entered, peak flow uses override directly.</t>
+          <t>Peak uses larger of average-based peaking method and cafeteria DFU-based equivalent.</t>
         </is>
       </c>
       <c r="E7" s="37" t="inlineStr">
@@ -3543,9 +4049,65 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="21" customHeight="1" s="32"/>
-    <row r="41" ht="21" customHeight="1" s="32"/>
-    <row r="42" ht="21" customHeight="1" s="32"/>
+    <row r="40" ht="21" customHeight="1" s="32">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>Cafeteria average flow (occupancy-based)</t>
+        </is>
+      </c>
+      <c r="B40" s="45">
+        <f>Inputs!B63</f>
+        <v/>
+      </c>
+      <c r="C40" s="37" t="inlineStr">
+        <is>
+          <t>m3/d</t>
+        </is>
+      </c>
+      <c r="D40" s="31" t="inlineStr">
+        <is>
+          <t>From cafeteria area, occupant factor, and unit wastewater flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="21" customHeight="1" s="32">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>Cafeteria equivalent peak flow (DFU-based)</t>
+        </is>
+      </c>
+      <c r="B41" s="45">
+        <f>Inputs!B61</f>
+        <v/>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>L/s</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>From estimated fixtures and DFU conversion; used as peak check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="21" customHeight="1" s="32">
+      <c r="A42" s="37" t="inlineStr">
+        <is>
+          <t>Cafeteria fixtures sanity check</t>
+        </is>
+      </c>
+      <c r="B42" s="45">
+        <f>IF(Inputs!B38&lt;=0,"No cafeteria area entered",IF(OR(Inputs!B45&lt;=0,Inputs!B46&lt;=0,Inputs!B48&lt;=0),"Complete cafeteria criteria",IF(Inputs!B58&gt;0,"Cafeteria module active","Check cafeteria inputs")))</f>
+        <v/>
+      </c>
+      <c r="C42" s="37" t="n"/>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>Confirm required fixture counts with architect/code consultant and AHJ.</t>
+        </is>
+      </c>
+    </row>
     <row r="43" ht="21" customHeight="1" s="32"/>
     <row r="44" ht="21" customHeight="1" s="32"/>
     <row r="45" ht="21" customHeight="1" s="32"/>
@@ -5082,6 +5644,7 @@
     <row r="79" ht="21" customHeight="1" s="32"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="N20:P20"/>
     <mergeCell ref="H7:L14"/>
     <mergeCell ref="T19:V19"/>
     <mergeCell ref="B7:F14"/>
@@ -5091,10 +5654,9 @@
     <mergeCell ref="N18:P18"/>
     <mergeCell ref="N22:P22"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H17:J17"/>
     <mergeCell ref="T17:V17"/>
     <mergeCell ref="T21:V21"/>
-    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="H17:J17"/>
     <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>